<commit_message>
Weekly refresh: Nike 2026-10-05
</commit_message>
<xml_diff>
--- a/examples/nike/latest/NKE_valuation_model.xlsx
+++ b/examples/nike/latest/NKE_valuation_model.xlsx
@@ -11115,7 +11115,7 @@
         </is>
       </c>
       <c r="C12" s="16" t="n">
-        <v>8.743692989132633</v>
+        <v>8.574907795821547</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -11167,7 +11167,7 @@
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>33.86999893188477</v>
+        <v>33.1150016784668</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
@@ -13021,17 +13021,17 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>0.9978029201690078</v>
+        <v>0.9980809582274758</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>0.1734704785408812</v>
+        <v>0.1731605706395805</v>
       </c>
       <c r="E5" s="29">
         <f>IF(C5="","",0.67*C5+0.33)</f>
         <v/>
       </c>
       <c r="F5" s="20" t="n">
-        <v>50269.85241470337</v>
+        <v>49149.28549118042</v>
       </c>
       <c r="G5" s="20" t="n">
         <v>7893</v>
@@ -13057,17 +13057,17 @@
         </is>
       </c>
       <c r="C6" s="28" t="n">
-        <v>1.107479456216676</v>
+        <v>1.101943304662855</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>0.1238911515970135</v>
+        <v>0.1227298182950117</v>
       </c>
       <c r="E6" s="29">
         <f>IF(C6="","",0.67*C6+0.33)</f>
         <v/>
       </c>
       <c r="F6" s="20" t="n">
-        <v>9974.415188765746</v>
+        <v>9680.863819744751</v>
       </c>
       <c r="G6" s="20" t="n">
         <v>0</v>
@@ -13093,17 +13093,17 @@
         </is>
       </c>
       <c r="C7" s="28" t="n">
-        <v>1.332130086461339</v>
+        <v>1.339563943850773</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0.1957824230000713</v>
+        <v>0.1980335502817881</v>
       </c>
       <c r="E7" s="29">
         <f>IF(C7="","",0.67*C7+0.33)</f>
         <v/>
       </c>
       <c r="F7" s="20" t="n">
-        <v>10793.09401491287</v>
+        <v>10823.78700783627</v>
       </c>
       <c r="G7" s="20" t="n">
         <v>0</v>
@@ -13129,17 +13129,17 @@
         </is>
       </c>
       <c r="C8" s="28" t="n">
-        <v>0.7795405742565485</v>
+        <v>0.7839976631019325</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>0.05868166593299189</v>
+        <v>0.0593018036572628</v>
       </c>
       <c r="E8" s="29">
         <f>IF(C8="","",0.67*C8+0.33)</f>
         <v/>
       </c>
       <c r="F8" s="20" t="n">
-        <v>5661.833731169892</v>
+        <v>5675.498253125</v>
       </c>
       <c r="G8" s="20" t="n">
         <v>1334</v>
@@ -13165,17 +13165,17 @@
         </is>
       </c>
       <c r="C9" s="28" t="n">
-        <v>0.992851435046608</v>
+        <v>1.00463607390288</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>0.08488357973844188</v>
+        <v>0.08723558488266825</v>
       </c>
       <c r="E9" s="29">
         <f>IF(C9="","",0.67*C9+0.33)</f>
         <v/>
       </c>
       <c r="F9" s="20" t="n">
-        <v>2034.423286477089</v>
+        <v>1982.633942303181</v>
       </c>
       <c r="G9" s="20" t="n">
         <v>591.158</v>
@@ -13201,17 +13201,17 @@
         </is>
       </c>
       <c r="C10" s="28" t="n">
-        <v>1.834634164867873</v>
+        <v>1.845813982374391</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>0.2355046167002563</v>
+        <v>0.2387257485618952</v>
       </c>
       <c r="E10" s="29">
         <f>IF(C10="","",0.67*C10+0.33)</f>
         <v/>
       </c>
       <c r="F10" s="20" t="n">
-        <v>5614.059842760344</v>
+        <v>5529.829296406031</v>
       </c>
       <c r="G10" s="20" t="n">
         <v>3530.009</v>
@@ -13237,17 +13237,17 @@
         </is>
       </c>
       <c r="C11" s="28" t="n">
-        <v>0.6312520892181978</v>
+        <v>0.6368901166498918</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>0.07539003600288942</v>
+        <v>0.07678802066229973</v>
       </c>
       <c r="E11" s="29">
         <f>IF(C11="","",0.67*C11+0.33)</f>
         <v/>
       </c>
       <c r="F11" s="20" t="n">
-        <v>2931.834243814385</v>
+        <v>2887.296219714615</v>
       </c>
       <c r="G11" s="20" t="n">
         <v>0</v>
@@ -14729,7 +14729,7 @@
         <v>2025</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>94.45999908447266</v>
+        <v>91.68000030517578</v>
       </c>
       <c r="F5" s="19" t="n">
         <v>105.594064</v>
@@ -14788,7 +14788,7 @@
         <v>2026</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>79.12000274658203</v>
+        <v>79.34500122070312</v>
       </c>
       <c r="F6" s="19" t="n">
         <v>136.414227</v>
@@ -14847,7 +14847,7 @@
         <v>2025</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>118.0899963378906</v>
+        <v>118.375</v>
       </c>
       <c r="F7" s="19" t="n">
         <v>47.945075</v>
@@ -14906,7 +14906,7 @@
         <v>2026</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>4.710000038146973</v>
+        <v>4.590099811553955</v>
       </c>
       <c r="F8" s="19" t="n">
         <v>431.937</v>
@@ -14965,7 +14965,7 @@
         <v>2026</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>14.32999992370605</v>
+        <v>14.11499977111816</v>
       </c>
       <c r="F9" s="19" t="n">
         <v>391.769705</v>
@@ -15024,7 +15024,7 @@
         <v>2025</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>57.27000045776367</v>
+        <v>56.40000152587891</v>
       </c>
       <c r="F10" s="19" t="n">
         <v>51.193194</v>
@@ -15083,7 +15083,7 @@
         <v>2026</v>
       </c>
       <c r="E11" s="47" t="n">
-        <v>33.86999893188477</v>
+        <v>33.1150016784668</v>
       </c>
       <c r="F11" s="48" t="n">
         <v>1484.2</v>
@@ -15359,10 +15359,10 @@
         </is>
       </c>
       <c r="C5" s="18" t="n">
-        <v>33.86999893188477</v>
+        <v>33.1150016784668</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>71.93000030517578</v>
+        <v>71.16999816894531</v>
       </c>
       <c r="E5" s="55">
         <f>IFERROR((C5+D5)/2,"")</f>
@@ -15535,10 +15535,10 @@
         </is>
       </c>
       <c r="C10" s="18" t="n">
-        <v>22.50271277839023</v>
+        <v>22.50137093614347</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>58.53136221653827</v>
+        <v>58.52582848659845</v>
       </c>
       <c r="E10" s="55">
         <f>IFERROR((C10+D10)/2,"")</f>
@@ -15737,7 +15737,7 @@
         </is>
       </c>
       <c r="C24" s="18" t="n">
-        <v>22.50271277839023</v>
+        <v>22.50137093614347</v>
       </c>
       <c r="D24" s="26">
         <f>C24/$C$18-1</f>
@@ -15751,7 +15751,7 @@
         </is>
       </c>
       <c r="C25" s="18" t="n">
-        <v>35.57076886190443</v>
+        <v>35.56816024949952</v>
       </c>
       <c r="D25" s="26">
         <f>C25/$C$18-1</f>
@@ -15765,7 +15765,7 @@
         </is>
       </c>
       <c r="C26" s="18" t="n">
-        <v>58.53136221653827</v>
+        <v>58.52582848659845</v>
       </c>
       <c r="D26" s="26">
         <f>C26/$C$18-1</f>

</xml_diff>

<commit_message>
Weekly refresh: Nike 2026-10-12
</commit_message>
<xml_diff>
--- a/examples/nike/latest/NKE_valuation_model.xlsx
+++ b/examples/nike/latest/NKE_valuation_model.xlsx
@@ -807,7 +807,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Rubber &amp; Plastics Footwear · fiscal year ends 05/31 · model date 2026-10-05 · Abhishek Raut</t>
+          <t>Rubber &amp; Plastics Footwear · fiscal year ends 05/31 · model date 2026-10-12 · Abhishek Raut</t>
         </is>
       </c>
     </row>
@@ -11040,11 +11040,11 @@
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>0.0524</v>
+        <v>0.0522</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>FRED DGS10 (10-year Treasury), 2026-10-01</t>
+          <t>FRED DGS10 (10-year Treasury), 2026-10-08</t>
         </is>
       </c>
     </row>
@@ -11115,7 +11115,7 @@
         </is>
       </c>
       <c r="C12" s="16" t="n">
-        <v>8.574907795821547</v>
+        <v>8.565206893386181</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -11167,11 +11167,11 @@
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>33.1150016784668</v>
+        <v>35.05500030517578</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Latest close, 2026-10-05.</t>
+          <t>Latest close, 2026-10-12.</t>
         </is>
       </c>
     </row>
@@ -13021,17 +13021,17 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>0.9980809582274758</v>
+        <v>1.000101116638327</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>0.1731605706395805</v>
+        <v>0.1735313454490617</v>
       </c>
       <c r="E5" s="29">
         <f>IF(C5="","",0.67*C5+0.33)</f>
         <v/>
       </c>
       <c r="F5" s="20" t="n">
-        <v>49149.28549118042</v>
+        <v>52028.6314529419</v>
       </c>
       <c r="G5" s="20" t="n">
         <v>7893</v>
@@ -13057,17 +13057,17 @@
         </is>
       </c>
       <c r="C6" s="28" t="n">
-        <v>1.101943304662855</v>
+        <v>1.095372923848844</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>0.1227298182950117</v>
+        <v>0.1223865607397181</v>
       </c>
       <c r="E6" s="29">
         <f>IF(C6="","",0.67*C6+0.33)</f>
         <v/>
       </c>
       <c r="F6" s="20" t="n">
-        <v>9680.863819744751</v>
+        <v>9955.936710937012</v>
       </c>
       <c r="G6" s="20" t="n">
         <v>0</v>
@@ -13093,17 +13093,17 @@
         </is>
       </c>
       <c r="C7" s="28" t="n">
-        <v>1.339563943850773</v>
+        <v>1.346027840923903</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>0.1980335502817881</v>
+        <v>0.1988067873819643</v>
       </c>
       <c r="E7" s="29">
         <f>IF(C7="","",0.67*C7+0.33)</f>
         <v/>
       </c>
       <c r="F7" s="20" t="n">
-        <v>10823.78700783627</v>
+        <v>11395.70327986091</v>
       </c>
       <c r="G7" s="20" t="n">
         <v>0</v>
@@ -13129,17 +13129,17 @@
         </is>
       </c>
       <c r="C8" s="28" t="n">
-        <v>0.7839976631019325</v>
+        <v>0.7766122136704851</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>0.0593018036572628</v>
+        <v>0.05808673940725519</v>
       </c>
       <c r="E8" s="29">
         <f>IF(C8="","",0.67*C8+0.33)</f>
         <v/>
       </c>
       <c r="F8" s="20" t="n">
-        <v>5675.498253125</v>
+        <v>5651.765309314918</v>
       </c>
       <c r="G8" s="20" t="n">
         <v>1334</v>
@@ -13165,17 +13165,17 @@
         </is>
       </c>
       <c r="C9" s="28" t="n">
-        <v>1.00463607390288</v>
+        <v>0.9970651775670069</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>0.08723558488266825</v>
+        <v>0.08857007780821731</v>
       </c>
       <c r="E9" s="29">
         <f>IF(C9="","",0.67*C9+0.33)</f>
         <v/>
       </c>
       <c r="F9" s="20" t="n">
-        <v>1982.633942303181</v>
+        <v>2133.768804715633</v>
       </c>
       <c r="G9" s="20" t="n">
         <v>591.158</v>
@@ -13201,17 +13201,17 @@
         </is>
       </c>
       <c r="C10" s="28" t="n">
-        <v>1.845813982374391</v>
+        <v>1.853907555195999</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>0.2387257485618952</v>
+        <v>0.2399399971835262</v>
       </c>
       <c r="E10" s="29">
         <f>IF(C10="","",0.67*C10+0.33)</f>
         <v/>
       </c>
       <c r="F10" s="20" t="n">
-        <v>5529.829296406031</v>
+        <v>6176.249533828454</v>
       </c>
       <c r="G10" s="20" t="n">
         <v>3530.009</v>
@@ -13237,17 +13237,17 @@
         </is>
       </c>
       <c r="C11" s="28" t="n">
-        <v>0.6368901166498918</v>
+        <v>0.629895039993271</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>0.07678802066229973</v>
+        <v>0.0762082382206922</v>
       </c>
       <c r="E11" s="29">
         <f>IF(C11="","",0.67*C11+0.33)</f>
         <v/>
       </c>
       <c r="F11" s="20" t="n">
-        <v>2887.296219714615</v>
+        <v>2884.736403785385</v>
       </c>
       <c r="G11" s="20" t="n">
         <v>0</v>
@@ -14729,7 +14729,7 @@
         <v>2025</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>91.68000030517578</v>
+        <v>94.28500366210938</v>
       </c>
       <c r="F5" s="19" t="n">
         <v>105.594064</v>
@@ -14788,7 +14788,7 @@
         <v>2026</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>79.34500122070312</v>
+        <v>83.53749847412109</v>
       </c>
       <c r="F6" s="19" t="n">
         <v>136.414227</v>
@@ -14847,7 +14847,7 @@
         <v>2025</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>118.375</v>
+        <v>117.879997253418</v>
       </c>
       <c r="F7" s="19" t="n">
         <v>47.945075</v>
@@ -14906,7 +14906,7 @@
         <v>2026</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>4.590099811553955</v>
+        <v>4.940000057220459</v>
       </c>
       <c r="F8" s="19" t="n">
         <v>431.937</v>
@@ -14965,7 +14965,7 @@
         <v>2026</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>14.11499977111816</v>
+        <v>15.76500034332275</v>
       </c>
       <c r="F9" s="19" t="n">
         <v>391.769705</v>
@@ -15024,7 +15024,7 @@
         <v>2025</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>56.40000152587891</v>
+        <v>56.34999847412109</v>
       </c>
       <c r="F10" s="19" t="n">
         <v>51.193194</v>
@@ -15083,7 +15083,7 @@
         <v>2026</v>
       </c>
       <c r="E11" s="47" t="n">
-        <v>33.1150016784668</v>
+        <v>35.05500030517578</v>
       </c>
       <c r="F11" s="48" t="n">
         <v>1484.2</v>
@@ -15359,10 +15359,10 @@
         </is>
       </c>
       <c r="C5" s="18" t="n">
-        <v>33.1150016784668</v>
+        <v>33.86999893188477</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>71.16999816894531</v>
+        <v>69.68000030517578</v>
       </c>
       <c r="E5" s="55">
         <f>IFERROR((C5+D5)/2,"")</f>
@@ -15535,10 +15535,10 @@
         </is>
       </c>
       <c r="C10" s="18" t="n">
-        <v>22.50137093614347</v>
+        <v>22.45254984251579</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>58.52582848659845</v>
+        <v>58.32474090200481</v>
       </c>
       <c r="E10" s="55">
         <f>IFERROR((C10+D10)/2,"")</f>
@@ -15737,7 +15737,7 @@
         </is>
       </c>
       <c r="C24" s="18" t="n">
-        <v>22.50137093614347</v>
+        <v>22.45254984251579</v>
       </c>
       <c r="D24" s="26">
         <f>C24/$C$18-1</f>
@@ -15751,7 +15751,7 @@
         </is>
       </c>
       <c r="C25" s="18" t="n">
-        <v>35.56816024949952</v>
+        <v>35.47329512205818</v>
       </c>
       <c r="D25" s="26">
         <f>C25/$C$18-1</f>
@@ -15765,7 +15765,7 @@
         </is>
       </c>
       <c r="C26" s="18" t="n">
-        <v>58.52582848659845</v>
+        <v>58.32474090200481</v>
       </c>
       <c r="D26" s="26">
         <f>C26/$C$18-1</f>

</xml_diff>